<commit_message>
le commit du lundi-1
</commit_message>
<xml_diff>
--- a/backend/data/modele_import_rwa.xlsx
+++ b/backend/data/modele_import_rwa.xlsx
@@ -23,11 +23,10 @@
     <sheet name="(j) créances à risque élevé" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="(k) autres actifs" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="(l) Hors bilan" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Feuil2" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Mapping des pondérations" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Ref_Ponderation" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Guide" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Listes (completees)" sheetId="22" state="hidden" r:id="rId22"/>
+    <sheet name="Mapping des pondérations" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Ref_Ponderation" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Guide" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Listes (completees)" sheetId="21" state="hidden" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="LISTCRM">LISTE!$G$3:$G$4</definedName>
@@ -1032,7 +1031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA19"/>
+  <dimension ref="A1:BG19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="30.6328125" defaultRowHeight="24" customHeight="1"/>
   <cols>
     <col width="18.26953125" customWidth="1" style="3" min="1" max="1"/>
@@ -1087,6 +1086,12 @@
     <col width="38" customWidth="1" style="173" min="51" max="51"/>
     <col width="37" customWidth="1" style="173" min="52" max="52"/>
     <col width="38" customWidth="1" style="173" min="53" max="53"/>
+    <col width="22" customWidth="1" style="173" min="54" max="54"/>
+    <col width="20" customWidth="1" style="173" min="55" max="55"/>
+    <col width="23" customWidth="1" style="173" min="56" max="56"/>
+    <col width="29" customWidth="1" style="173" min="57" max="57"/>
+    <col width="18" customWidth="1" style="173" min="58" max="58"/>
+    <col width="16" customWidth="1" style="173" min="59" max="59"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" s="173">
@@ -1353,6 +1358,36 @@
       <c r="BA1" s="174" t="inlineStr">
         <is>
           <t>Entreprise_investissement_hors_loi_bancaire</t>
+        </is>
+      </c>
+      <c r="BB1" s="174" t="inlineStr">
+        <is>
+          <t>N_Centrale_risques</t>
+        </is>
+      </c>
+      <c r="BC1" s="174" t="inlineStr">
+        <is>
+          <t>Secteur_activite</t>
+        </is>
+      </c>
+      <c r="BD1" s="174" t="inlineStr">
+        <is>
+          <t>Groupe_clients_lies</t>
+        </is>
+      </c>
+      <c r="BE1" s="174" t="inlineStr">
+        <is>
+          <t>N_Centrale_risques_groupe</t>
+        </is>
+      </c>
+      <c r="BF1" s="174" t="inlineStr">
+        <is>
+          <t>Categorie_lien</t>
+        </is>
+      </c>
+      <c r="BG1" s="174" t="inlineStr">
+        <is>
+          <t>Partie_liee</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3822,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="10">
+  <dataValidations count="13">
     <dataValidation sqref="R2:R19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"OUI, NON"</formula1>
     </dataValidation>
@@ -3818,6 +3853,15 @@
     <dataValidation sqref="AV2:AV2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste deroulante pour que le calcul prudentiel s'applique a cette ligne." type="list">
       <formula1>"0.2,0.35,0.5,0.75,1.0,1.5,2.5"</formula1>
     </dataValidation>
+    <dataValidation sqref="BC2:BC2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste deroulante pour que le calcul prudentiel s'applique a cette ligne." type="list">
+      <formula1>'Listes (completees)'!$C$3:$C$23</formula1>
+    </dataValidation>
+    <dataValidation sqref="BF2:BF2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste deroulante pour que le calcul prudentiel s'applique a cette ligne." type="list">
+      <formula1>"Controle de droit,Controle de fait,Dependance economique"</formula1>
+    </dataValidation>
+    <dataValidation sqref="BG2:BG2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste deroulante pour que le calcul prudentiel s'applique a cette ligne." type="list">
+      <formula1>"Actionnaire detenant au moins 10 %,Membre de l'organe deliberant,Membre de l'organe executif,Commissaire aux comptes,Personnel de direction,Cadre moyen ou superieur,Personnel d'execution,Autre partie liee"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4811,7 +4855,6 @@
       </c>
       <c r="B1" s="90" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="92" t="inlineStr">
         <is>
@@ -5421,136 +5464,6 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="C2:E9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="48.453125" customWidth="1" style="173" min="3" max="3"/>
-    <col width="53.81640625" customWidth="1" style="173" min="4" max="4"/>
-    <col width="103.90625" customWidth="1" style="173" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="23.5" customHeight="1" s="173">
-      <c r="C2" s="162" t="inlineStr">
-        <is>
-          <t>Hors - Bilan</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="29.5" customHeight="1" s="173">
-      <c r="C4" s="161" t="inlineStr">
-        <is>
-          <t>Niveau de risque(à mettre dans le selecteur)</t>
-        </is>
-      </c>
-      <c r="D4" s="161" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Facteur de Conversion en Equivalent Crédit (FCEC)</t>
-        </is>
-      </c>
-      <c r="E4" s="161" t="inlineStr">
-        <is>
-          <t>Elements hors bilan concernés(à mettre dans une icone info pour etre consultées au survol de la souris)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="28.5" customHeight="1" s="173">
-      <c r="C5" s="158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Risque flaible </t>
-        </is>
-      </c>
-      <c r="D5" s="109" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E5" s="160" t="inlineStr">
-        <is>
-          <t xml:space="preserve">*Engagements révocables sans condition (à tout moment, sans préavis ou caducs automatiquement)
-</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42.5" customHeight="1" s="173">
-      <c r="C6" s="110" t="inlineStr">
-        <is>
-          <t>Risque mineur</t>
-        </is>
-      </c>
-      <c r="D6" s="111" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E6" s="164" t="inlineStr">
-        <is>
-          <t xml:space="preserve">*Engagements ≤ 1 an non révocables sans condition
-*Lettres de crédit commerciales à court terme (crédits documentaires)
-</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="42.5" customHeight="1" s="173">
-      <c r="C7" s="108" t="inlineStr">
-        <is>
-          <t>Risque moyen</t>
-        </is>
-      </c>
-      <c r="D7" s="109" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E7" s="160" t="inlineStr">
-        <is>
-          <t>*Engagements &gt; 1 an non révocables sans condition
-*Lettres de crédit documentaires non garanties par marchandises
-*Garanties de bonne exécution, de soumission, de tiers, crédits de confirmation</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="56.5" customHeight="1" s="173">
-      <c r="C8" s="110" t="inlineStr">
-        <is>
-          <t>Risque élevé</t>
-        </is>
-      </c>
-      <c r="D8" s="111" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E8" s="164" t="inlineStr">
-        <is>
-          <t xml:space="preserve">*Facilités d’émission d’effets (FEE) et facilités de prise ferme renouvelables (FPR)
-*Substituts directs de crédit (garanties d’endettement, acceptations…)
-</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="84.5" customHeight="1" s="173">
-      <c r="C9" s="108" t="inlineStr">
-        <is>
-          <t>Risque très élevé</t>
-        </is>
-      </c>
-      <c r="D9" s="163" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="160" t="inlineStr">
-        <is>
-          <t xml:space="preserve">*Opérations assimilables à des pensions (repo / prêts de titres)
-*Cessions d’actifs avec recours (affacturage, escompte…)
-*Engagements d’achat d’actifs à terme / dépôts à terme contre terme
-*Fraction non versée d’actions / titres partiellement libérés
-*Autres éléments hors bilan non classés
-</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Feuil18">
     <tabColor rgb="FF66FFFF"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5835,6 +5748,1096 @@
       <c r="C15" s="122" t="n"/>
       <c r="D15" s="122" t="n"/>
       <c r="E15" s="122" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr codeName="Feuil19">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:W20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="14" customWidth="1" style="173" min="1" max="17"/>
+    <col width="34" customWidth="1" style="173" min="19" max="20"/>
+    <col width="28.1796875" customWidth="1" style="173" min="23" max="23"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="128" t="inlineStr">
+        <is>
+          <t>Table de paramètres pour Excel web</t>
+        </is>
+      </c>
+      <c r="B1" s="128" t="n"/>
+      <c r="C1" s="128" t="n"/>
+      <c r="D1" s="128" t="n"/>
+      <c r="E1" s="128" t="n"/>
+      <c r="F1" s="128" t="n"/>
+      <c r="G1" s="128" t="n"/>
+      <c r="H1" s="128" t="n"/>
+      <c r="I1" s="128" t="n"/>
+      <c r="J1" s="128" t="n"/>
+      <c r="K1" s="128" t="n"/>
+      <c r="L1" s="128" t="n"/>
+      <c r="M1" s="128" t="n"/>
+      <c r="N1" s="128" t="n"/>
+      <c r="O1" s="128" t="n"/>
+      <c r="P1" s="128" t="n"/>
+      <c r="Q1" s="128" t="n"/>
+      <c r="S1" s="128" t="inlineStr">
+        <is>
+          <t>(a) souverains</t>
+        </is>
+      </c>
+      <c r="T1" s="128" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="W1" s="142" t="inlineStr">
+        <is>
+          <t>(a) souverains</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="128" t="inlineStr">
+        <is>
+          <t>Notation_norm</t>
+        </is>
+      </c>
+      <c r="B2" s="128" t="inlineStr">
+        <is>
+          <t>RW_souverain</t>
+        </is>
+      </c>
+      <c r="C2" s="128" t="n"/>
+      <c r="D2" s="128" t="inlineStr">
+        <is>
+          <t>Notation_norm</t>
+        </is>
+      </c>
+      <c r="E2" s="128" t="inlineStr">
+        <is>
+          <t>RW_org_pub</t>
+        </is>
+      </c>
+      <c r="F2" s="128" t="n"/>
+      <c r="G2" s="128" t="inlineStr">
+        <is>
+          <t>Notation_norm</t>
+        </is>
+      </c>
+      <c r="H2" s="128" t="inlineStr">
+        <is>
+          <t>RW_entreprise</t>
+        </is>
+      </c>
+      <c r="I2" s="128" t="n"/>
+      <c r="J2" s="128" t="inlineStr">
+        <is>
+          <t>Notation_norm</t>
+        </is>
+      </c>
+      <c r="K2" s="128" t="inlineStr">
+        <is>
+          <t>RW_inst_&lt;=3m</t>
+        </is>
+      </c>
+      <c r="L2" s="128" t="n"/>
+      <c r="M2" s="128" t="inlineStr">
+        <is>
+          <t>Notation_norm</t>
+        </is>
+      </c>
+      <c r="N2" s="128" t="inlineStr">
+        <is>
+          <t>RW_inst_&gt;3m</t>
+        </is>
+      </c>
+      <c r="O2" s="128" t="n"/>
+      <c r="P2" s="128" t="inlineStr">
+        <is>
+          <t>Type_HB</t>
+        </is>
+      </c>
+      <c r="Q2" s="128" t="inlineStr">
+        <is>
+          <t>CCF_HB</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>(b) organismes pub. hors Adm c</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>AA+</t>
+        </is>
+      </c>
+      <c r="W2" s="130" t="inlineStr">
+        <is>
+          <t>(b) organismes pub. hors Adm c</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Risque faible</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>(c) Expositions sur les BMD</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="W3" s="130" t="inlineStr">
+        <is>
+          <t>(c) BMD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AA+</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AA+</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>AA+</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>AA+</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>AA+</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Risque mineur</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>(d) institutions financières</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="W4" s="130" t="inlineStr">
+        <is>
+          <t>(d) institutions financières</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Risque moyen</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>(e) entreprises</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="W5" s="130" t="inlineStr">
+        <is>
+          <t>(e) entreprises</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Risque élevé</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>(f) clientèle de détail</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W6" s="130" t="inlineStr">
+        <is>
+          <t>(f) clientèle de détail</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>A+</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Risque très élevé</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>(g) prêts garantis par l'immo R</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="W7" s="130" t="inlineStr">
+        <is>
+          <t>(k) autres actifs</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>(h) prêts garantis par l'immo C</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>BBB+</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>(i) créances en souffrance</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BBB+</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>BBB+</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>BBB+</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>BBB+</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>BBB+</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>(j) créances à risque élevé</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>(k) autres actifs</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>BB+</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>(l) Hors bilan</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BB+</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>BB+</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>BB+</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>BB+</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>BB+</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>BB-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BB-</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>BB-</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>BB-</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>BB-</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>BB-</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>1</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>&lt; B-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>1</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Non noté</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>&lt; B-</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>&lt; B-</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>&lt; B-</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>&lt; B-</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>&lt; B-</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Non noté</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Non noté</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Non noté</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Non noté</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>1</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Non noté</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7062,1096 +8065,6 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr codeName="Feuil19">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:W20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="14" customWidth="1" style="173" min="1" max="17"/>
-    <col width="34" customWidth="1" style="173" min="19" max="20"/>
-    <col width="28.1796875" customWidth="1" style="173" min="23" max="23"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="128" t="inlineStr">
-        <is>
-          <t>Table de paramètres pour Excel web</t>
-        </is>
-      </c>
-      <c r="B1" s="128" t="n"/>
-      <c r="C1" s="128" t="n"/>
-      <c r="D1" s="128" t="n"/>
-      <c r="E1" s="128" t="n"/>
-      <c r="F1" s="128" t="n"/>
-      <c r="G1" s="128" t="n"/>
-      <c r="H1" s="128" t="n"/>
-      <c r="I1" s="128" t="n"/>
-      <c r="J1" s="128" t="n"/>
-      <c r="K1" s="128" t="n"/>
-      <c r="L1" s="128" t="n"/>
-      <c r="M1" s="128" t="n"/>
-      <c r="N1" s="128" t="n"/>
-      <c r="O1" s="128" t="n"/>
-      <c r="P1" s="128" t="n"/>
-      <c r="Q1" s="128" t="n"/>
-      <c r="S1" s="128" t="inlineStr">
-        <is>
-          <t>(a) souverains</t>
-        </is>
-      </c>
-      <c r="T1" s="128" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="W1" s="142" t="inlineStr">
-        <is>
-          <t>(a) souverains</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="128" t="inlineStr">
-        <is>
-          <t>Notation_norm</t>
-        </is>
-      </c>
-      <c r="B2" s="128" t="inlineStr">
-        <is>
-          <t>RW_souverain</t>
-        </is>
-      </c>
-      <c r="C2" s="128" t="n"/>
-      <c r="D2" s="128" t="inlineStr">
-        <is>
-          <t>Notation_norm</t>
-        </is>
-      </c>
-      <c r="E2" s="128" t="inlineStr">
-        <is>
-          <t>RW_org_pub</t>
-        </is>
-      </c>
-      <c r="F2" s="128" t="n"/>
-      <c r="G2" s="128" t="inlineStr">
-        <is>
-          <t>Notation_norm</t>
-        </is>
-      </c>
-      <c r="H2" s="128" t="inlineStr">
-        <is>
-          <t>RW_entreprise</t>
-        </is>
-      </c>
-      <c r="I2" s="128" t="n"/>
-      <c r="J2" s="128" t="inlineStr">
-        <is>
-          <t>Notation_norm</t>
-        </is>
-      </c>
-      <c r="K2" s="128" t="inlineStr">
-        <is>
-          <t>RW_inst_&lt;=3m</t>
-        </is>
-      </c>
-      <c r="L2" s="128" t="n"/>
-      <c r="M2" s="128" t="inlineStr">
-        <is>
-          <t>Notation_norm</t>
-        </is>
-      </c>
-      <c r="N2" s="128" t="inlineStr">
-        <is>
-          <t>RW_inst_&gt;3m</t>
-        </is>
-      </c>
-      <c r="O2" s="128" t="n"/>
-      <c r="P2" s="128" t="inlineStr">
-        <is>
-          <t>Type_HB</t>
-        </is>
-      </c>
-      <c r="Q2" s="128" t="inlineStr">
-        <is>
-          <t>CCF_HB</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>(b) organismes pub. hors Adm c</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>AA+</t>
-        </is>
-      </c>
-      <c r="W2" s="130" t="inlineStr">
-        <is>
-          <t>(b) organismes pub. hors Adm c</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Risque faible</t>
-        </is>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>(c) Expositions sur les BMD</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="W3" s="130" t="inlineStr">
-        <is>
-          <t>(c) BMD</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>AA+</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>AA+</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>AA+</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>AA+</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>AA+</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Risque mineur</t>
-        </is>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>(d) institutions financières</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>AA-</t>
-        </is>
-      </c>
-      <c r="W4" s="130" t="inlineStr">
-        <is>
-          <t>(d) institutions financières</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Risque moyen</t>
-        </is>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>(e) entreprises</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>A+</t>
-        </is>
-      </c>
-      <c r="W5" s="130" t="inlineStr">
-        <is>
-          <t>(e) entreprises</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AA-</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>AA-</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>AA-</t>
-        </is>
-      </c>
-      <c r="H6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>AA-</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>AA-</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Risque élevé</t>
-        </is>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>(f) clientèle de détail</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="W6" s="130" t="inlineStr">
-        <is>
-          <t>(f) clientèle de détail</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>A+</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>A+</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>A+</t>
-        </is>
-      </c>
-      <c r="H7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>A+</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>A+</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Risque très élevé</t>
-        </is>
-      </c>
-      <c r="Q7" t="n">
-        <v>1</v>
-      </c>
-      <c r="S7" t="inlineStr">
-        <is>
-          <t>(g) prêts garantis par l'immo R</t>
-        </is>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>A-</t>
-        </is>
-      </c>
-      <c r="W7" s="130" t="inlineStr">
-        <is>
-          <t>(k) autres actifs</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="S8" t="inlineStr">
-        <is>
-          <t>(h) prêts garantis par l'immo C</t>
-        </is>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>BBB+</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>A-</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>A-</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>A-</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>A-</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>A-</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>(i) créances en souffrance</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>BBB</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>BBB+</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>BBB+</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>BBB+</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>BBB+</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>BBB+</t>
-        </is>
-      </c>
-      <c r="N10" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>(j) créances à risque élevé</t>
-        </is>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>BBB</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>BBB</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>BBB</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>BBB</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>BBB</t>
-        </is>
-      </c>
-      <c r="N11" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>(k) autres actifs</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="S12" t="inlineStr">
-        <is>
-          <t>(l) Hors bilan</t>
-        </is>
-      </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-      <c r="N13" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="N14" t="n">
-        <v>1</v>
-      </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="N15" t="n">
-        <v>1</v>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="N16" t="n">
-        <v>1</v>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>1</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="N17" t="n">
-        <v>1</v>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>&lt; B-</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="N18" t="n">
-        <v>1</v>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>Non noté</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>&lt; B-</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>&lt; B-</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>&lt; B-</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>&lt; B-</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>&lt; B-</t>
-        </is>
-      </c>
-      <c r="N19" t="n">
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Non noté</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Non noté</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Non noté</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Non noté</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>1</v>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Non noté</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Feuil20">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -8270,13 +8183,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8297,6 +8210,11 @@
           <t>Type_Collatéral</t>
         </is>
       </c>
+      <c r="C2" s="177" t="inlineStr">
+        <is>
+          <t>Secteur_activite</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8309,6 +8227,11 @@
           <t>Liquidités dans la même devise</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Agriculture, elevage, sylviculture</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8321,6 +8244,11 @@
           <t>Liquidités dans une devise différente</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Peche et aquaculture</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8333,6 +8261,11 @@
           <t>Or</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Industries extractives</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8345,6 +8278,11 @@
           <t>Titre de dette souverain</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Industries manufacturieres</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8357,6 +8295,11 @@
           <t>Titre non noté émis par un État de l UMOA</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Agro-industrie</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8369,6 +8312,11 @@
           <t>Titre de dette émis par un autre émetteur</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Electricite, gaz et eau</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8381,6 +8329,11 @@
           <t>Titre garanti par un agent agréé par la BRVM</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Batiment et travaux publics</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8393,6 +8346,11 @@
           <t>Titre bancaire non noté</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Commerce de gros et de detail</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8405,6 +8363,11 @@
           <t>Action de l indice BRVM 10</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Transports et entreposage</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8417,6 +8380,11 @@
           <t>Action d un indice principal reconnu</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Hebergement et restauration</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8429,6 +8397,11 @@
           <t>Autre action cotée à la BRVM ou sur une bourse reconnue</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Information et communication</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8441,6 +8414,11 @@
           <t>Obligation convertible en action</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Activites financieres et d'assurance</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8453,6 +8431,11 @@
           <t>OPCVM / FI</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Activites immobilieres</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
@@ -8460,11 +8443,63 @@
           <t>Panier d actifs</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Activites specialisees, scientifiques et techniques</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
           <t>Autre sûreté non éligible</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Services administratifs et de soutien</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Administration publique</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Enseignement</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sante humaine et action sociale</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Arts, spectacles et loisirs</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Autres services</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Menages et particuliers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(import-fodep): validation des exigences conditionnelles et epuration des saisies FODEP sur l'ADPE
</commit_message>
<xml_diff>
--- a/backend/data/modele_import_rwa.xlsx
+++ b/backend/data/modele_import_rwa.xlsx
@@ -15,13 +15,7 @@
     <sheet name="Listes de référence" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="ListeCascade1">'Listes (validation)'!$W$2:$W$2</definedName>
-    <definedName name="ListeCascade2">'Listes (validation)'!$I$2:$I$13</definedName>
-    <definedName name="ListeCascade3">'Listes (validation)'!$A$2:$A$3</definedName>
-    <definedName name="ListeCascade4">'Listes (validation)'!$J$2:$J$9</definedName>
-    <definedName name="ListeCascade5">'Listes (validation)'!$K$2:$K$4</definedName>
-    <definedName name="ListeCascade6">'Listes (validation)'!$L$2:$L$14</definedName>
-    <definedName name="ListeCascade7">'Listes (validation)'!$P$2:$P$8</definedName>
+    <definedName name="ListeCascade1">'Listes (validation)'!$AB$2:$AB$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -100,12 +94,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
+        <fgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -152,14 +146,14 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -168,7 +162,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -378,107 +372,27 @@
     </comment>
     <comment ref="Z1" authorId="0" shapeId="0">
       <text>
-        <t>Optionnel — Type spécifique d'exposition souveraine (pondération préférentielle)</t>
+        <t>Optionnel — Régime ou traitement prudentiel spécifique au sens des circulaires BCEAO</t>
       </text>
     </comment>
     <comment ref="AA1" authorId="0" shapeId="0">
       <text>
-        <t>Optionnel — Souverain préférentiel à pondération nulle</t>
+        <t>Optionnel — Type spécifique d'exposition souveraine (pondération préférentielle)</t>
       </text>
     </comment>
     <comment ref="AB1" authorId="0" shapeId="0">
       <text>
-        <t>Optionnel — Souverain non noté établi par les OCE</t>
+        <t>Optionnel — Note OCE de 0 à 7</t>
       </text>
     </comment>
     <comment ref="AC1" authorId="0" shapeId="0">
       <text>
-        <t>Optionnel — Note OCE de 0 à 7</t>
+        <t>Optionnel — Type d'élément d'actif (catégorie autres actifs)</t>
       </text>
     </comment>
     <comment ref="AD1" authorId="0" shapeId="0">
       <text>
-        <t>Optionnel — Organisme public hors administration centrale, libellé et financé en FCFA</t>
-      </text>
-    </comment>
-    <comment ref="AE1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — L'organisme public finance une activité non publique</t>
-      </text>
-    </comment>
-    <comment ref="AF1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — BMD notation élevée / soutien actionnarial fort</t>
-      </text>
-    </comment>
-    <comment ref="AG1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — BMD relevant du cas UEMOA libellé et financé en FCFA</t>
-      </text>
-    </comment>
-    <comment ref="AH1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — BMD UEMOA en FCFA respectant les critères c), d) et e)</t>
-      </text>
-    </comment>
-    <comment ref="AI1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — BMD de la liste BIRD/SFI/BAsD/BAD/BERD/BEI/FEI/BNI/BDC/BIsD/BDCE/AMGI/BOAD</t>
-      </text>
-    </comment>
-    <comment ref="AJ1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Cas prudentiel des institutions bancaires</t>
-      </text>
-    </comment>
-    <comment ref="AK1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Type d'élément d'actif (catégorie autres actifs)</t>
-      </text>
-    </comment>
-    <comment ref="AL1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Critères de classement en clientèle de détail respectés</t>
-      </text>
-    </comment>
-    <comment ref="AM1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Conditions d'éligibilité de l'immobilier résidentiel respectées</t>
-      </text>
-    </comment>
-    <comment ref="AN1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Conditions d'éligibilité de l'immobilier commercial respectées</t>
-      </text>
-    </comment>
-    <comment ref="AO1" authorId="0" shapeId="0">
-      <text>
         <t>Optionnel — Pondération initiale de l'exposition avant défaut</t>
-      </text>
-    </comment>
-    <comment ref="AP1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Exposition en défaut = prêt immobilier résidentiel</t>
-      </text>
-    </comment>
-    <comment ref="AQ1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Provisions ≥ 20 % de l'encours</t>
-      </text>
-    </comment>
-    <comment ref="AR1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Portefeuille entreprises dépassant le seuil BCEAO de dégradation</t>
-      </text>
-    </comment>
-    <comment ref="AS1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Entreprise faisant l'objet d'une procédure prudentielle</t>
-      </text>
-    </comment>
-    <comment ref="AT1" authorId="0" shapeId="0">
-      <text>
-        <t>Optionnel — Entreprise d'investissement non soumise à la loi bancaire</t>
       </text>
     </comment>
   </commentList>
@@ -879,7 +793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W199"/>
+  <dimension ref="A1:AB199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
@@ -926,71 +840,96 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>Standard (aucun traitement particulier)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>Expositions sur États de l’UEMOA et démembrements libellées et financées en FCFA</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Organisme public standard (selon notation)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>BMD standard (selon notation)</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>equivalent_umoa_rules</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Prêt immobilier résidentiel en défaut (Provisions &gt;= 20%) — 50%</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Entreprise standard (selon notation ou 100%)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Encaisse</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Controle de droit</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Actionnaire detenant au moins 10 %</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Agriculture, elevage, sylviculture</t>
         </is>
       </c>
-      <c r="P2" t="n">
+      <c r="U2" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>Souverains</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>emprunteur souverain</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>&lt;=1 an</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>Liquidités dans la même devise</t>
         </is>
       </c>
-      <c r="V2" t="n">
+      <c r="AA2" t="n">
         <v>0</v>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>(Sans objet pour cette catégorie)</t>
         </is>
@@ -1039,68 +978,93 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>Souverain UEMOA en FCFA (pondération 0 %)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>Expositions sur BCEAO libellées et financées en FCFA</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Organisme public UEMOA libellé en FCFA (préférentiel 20%)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>BMD haute qualité / soutien fort (pondération 0%)</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
         <is>
           <t>weak_prudential_case</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Prêt immobilier résidentiel en défaut (Provisions &lt; 20%) — 100%</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Portefeuille dégradé (seuil BCEAO dépassé -&gt; 150%)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Valeurs assimilées à l’encaisse, y compris l’or</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Controle de fait</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>Membre de l'organe deliberant</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>Peche et aquaculture</t>
         </is>
       </c>
-      <c r="P3" t="n">
+      <c r="U3" t="n">
         <v>0.35</v>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>Organismes pub. hors Adm c</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>autre émetteur</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>AA+</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>1-3 ans</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>Liquidités dans une devise différente</t>
         </is>
       </c>
-      <c r="V3" t="n">
+      <c r="AA3" t="n">
         <v>0.005</v>
       </c>
     </row>
@@ -1142,63 +1106,88 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>Organisme public UEMOA en FCFA (pondération 20 %)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>UEMOA</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Activité commerciale / non publique (traité comme entreprise)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>BMD institution listée BCEAO en FCFA (BIRD, BAD, BOAD... 0%)</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>eligible_categories_case</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Autre créance en défaut (Provisions &gt;= 20%) — 100%</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Entreprise faisant l'objet d'une procédure prudentielle</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Valeurs à l’encaissement avec crédit immédiat</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Dependance economique</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Membre de l'organe executif</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Industries extractives</t>
         </is>
       </c>
-      <c r="P4" t="n">
+      <c r="U4" t="n">
         <v>0.5</v>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>Expositions sur les BMD</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>AA</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>3-5 ans</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>Or</t>
         </is>
       </c>
-      <c r="V4" t="n">
+      <c r="AA4" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -1230,53 +1219,73 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>Organisme public - Activité commerciale (traité comme entreprise)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>CEDEAO</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>BMD UEMOA en FCFA conforme aux critères (20%)</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Autre créance en défaut (Provisions &lt; 20%) — 150%</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Entreprise d'investissement non soumise à la loi bancaire (100%)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Participations non significatives non déduites des fonds propres</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>Commissaire aux comptes</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>Industries manufacturieres</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="U5" t="n">
         <v>0.75</v>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>Institutions financières</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>AA-</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>5-10 ans</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>Titre de dette souverain</t>
         </is>
       </c>
-      <c r="V5" t="n">
+      <c r="AA5" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -1308,53 +1317,58 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>BMD liste officielle BCEAO (BIRD, BAD, BOAD... pondération 0 %)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>UA</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Immobilisations corporelles</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>Personnel de direction</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>Agro-industrie</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="U6" t="n">
         <v>1</v>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>Entreprises</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>A+</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>&gt;10 ans</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>Titre non noté émis par un État de l UMOA</t>
         </is>
       </c>
-      <c r="V6" t="n">
+      <c r="AA6" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -1376,48 +1390,53 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>BMD haute qualité / soutien fort (pondération 0 %)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>UE</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Immobilisations hors exploitation</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Cadre moyen ou superieur</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>Electricite, gaz et eau</t>
         </is>
       </c>
-      <c r="P7" t="n">
+      <c r="U7" t="n">
         <v>1.5</v>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>Clientèle de détail</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>Titre de dette émis par un autre émetteur</t>
         </is>
       </c>
-      <c r="V7" t="n">
+      <c r="AA7" t="n">
         <v>0.04</v>
       </c>
     </row>
@@ -1439,48 +1458,53 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>BMD UEMOA en FCFA (pondération 20 %)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>ONU</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Immobilisations incorporelles</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Personnel d'execution</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>Batiment et travaux publics</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="U8" t="n">
         <v>2.5</v>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>Autres actifs</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>A-</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>Titre garanti par un agent agréé par la BRVM</t>
         </is>
       </c>
-      <c r="V8" t="n">
+      <c r="AA8" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -1502,40 +1526,45 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>Banque - Établissement de crédit agréé UEMOA</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>BRI</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>Autres actifs divers</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>Autre partie liee</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>Commerce de gros et de detail</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>BBB+</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>Titre bancaire non noté</t>
         </is>
       </c>
-      <c r="V9" t="n">
+      <c r="AA9" t="n">
         <v>0.09</v>
       </c>
     </row>
@@ -1557,30 +1586,35 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>Banque - Faible qualité prudentielle</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>FMI</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Engagements en actions non déduits</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>Transports et entreposage</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="X10" t="inlineStr">
         <is>
           <t>BBB</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>Action de l indice BRVM 10</t>
         </is>
       </c>
-      <c r="V10" t="n">
+      <c r="AA10" t="n">
         <v>0.12</v>
       </c>
     </row>
@@ -1602,30 +1636,35 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>Clientèle de détail - Critères d'éligibilité respectés (pondération 75 %)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>BCE</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Expositions sur entreprises financières non soumises à une réglementation équivalente UMOA</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>Hebergement et restauration</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>BBB-</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>Action d un indice principal reconnu</t>
         </is>
       </c>
-      <c r="V11" t="n">
+      <c r="AA11" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -1647,30 +1686,35 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>Immobilier résidentiel - Prêt éligible avec hypothèque 1er rang (pondération 35 %)</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>FGD-UMOA</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>Autres éléments d’actifs non définis</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>Information et communication</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>BB+</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="Z12" t="inlineStr">
         <is>
           <t>Autre action cotée à la BRVM ou sur une bourse reconnue</t>
         </is>
       </c>
-      <c r="V12" t="n">
+      <c r="AA12" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1687,30 +1731,35 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>Immobilier commercial - Prêt éligible (pondération 50 %)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>Aucun de ces cas</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>Participations significatives et impôts différés actifs non déduits</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>Activites financieres et d'assurance</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>BB</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="Z13" t="inlineStr">
         <is>
           <t>Obligation convertible en action</t>
         </is>
       </c>
-      <c r="V13" t="n">
+      <c r="AA13" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -1725,22 +1774,27 @@
           <t>Autriche</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Défaut - Prêt immobilier résidentiel (Provisions &gt;= 20%) — pondération 50 %</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
         <is>
           <t>Expositions sur établissements non conformes aux ratios de solvabilité</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>Activites immobilieres</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>BB-</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="Z14" t="inlineStr">
         <is>
           <t>OPCVM / FI</t>
         </is>
@@ -1757,17 +1811,22 @@
           <t>Azerbaidjan</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Défaut - Prêt immobilier résidentiel (Provisions &lt; 20%) — pondération 100 %</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
         <is>
           <t>Activites specialisees, scientifiques et techniques</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>&lt; B-</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="Z15" t="inlineStr">
         <is>
           <t>Panier d actifs</t>
         </is>
@@ -1784,17 +1843,22 @@
           <t>Bahamas</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Défaut - Autre créance en souffrance (Provisions &gt;= 20%) — pondération 100 %</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
         <is>
           <t>Services administratifs et de soutien</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>Non noté</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t>Autre sûreté non éligible</t>
         </is>
@@ -1811,7 +1875,12 @@
           <t>Bahrein</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Défaut - Autre créance en souffrance (Provisions &lt; 20%) — pondération 150 %</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
         <is>
           <t>Administration publique</t>
         </is>
@@ -1828,7 +1897,12 @@
           <t>Bangladesh</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Entreprise - Portefeuille dégradé (seuil BCEAO dépassé -&gt; pondération 150 %)</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
         <is>
           <t>Enseignement</t>
         </is>
@@ -1845,7 +1919,12 @@
           <t>Barbade</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Entreprise - Procédure prudentielle (pondération 150 %)</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
         <is>
           <t>Sante humaine et action sociale</t>
         </is>
@@ -1857,7 +1936,12 @@
           <t>Belgique</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Entreprise d'investissement non soumise à la loi bancaire (pondération 100 %)</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
         <is>
           <t>Arts, spectacles et loisirs</t>
         </is>
@@ -1869,7 +1953,7 @@
           <t>Belize</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>Autres services</t>
         </is>
@@ -1881,7 +1965,7 @@
           <t>Benin</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
+      <c r="T22" t="inlineStr">
         <is>
           <t>Menages et particuliers</t>
         </is>
@@ -3231,19 +3315,19 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Chaque colonne à choix (catégorie, notation, devise, pays, type de CRM, cas particuliers, champs Oui/Non...) propose une liste déroulante : cliquez sur la cellule puis sur la flèche qui apparaît pour choisir une valeur reconnue par le calcul. Le détail des valeurs figure aussi dans l'onglet « Listes de référence ».</t>
+          <t>Chaque colonne à choix (catégorie, notation, devise, pays, type de CRM, régime prudentiel spécifique...) propose une liste déroulante : cliquez sur la cellule puis sur la flèche qui apparaît pour choisir une valeur reconnue par le calcul. Le détail des valeurs figure aussi dans l'onglet « Listes de référence ».</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Listes en cascade</t>
+          <t>Régime prudentiel spécifique</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Comme dans le formulaire « Ajouter une exposition », certaines listes dépendent de la « Catégorie d'exposition » choisie sur la même ligne (ex. Cas_institution_bancaire ne propose des options que si la catégorie est Institutions financières, Type_autre_actif seulement pour Autres actifs, Cas_particulier_souverain et les champs Souverain_* seulement pour Souverains, etc.). Choisissez d'abord la catégorie : les colonnes qui ne la concernent pas n'affichent alors que « (Sans objet pour cette catégorie) », et se réactivent automatiquement si vous changez la catégorie.</t>
+          <t>La colonne « Regime_prudentiel_specifique » rassemble en une seule liste déroulante tous les cas et traitements particuliers de la réglementation BCEAO : taux préférentiels (Souverain UEMOA 0%, Prêt immobilier résidentiel 35%, Clientèle de détail 75%, BMD 0%), surpondérations (Défauts 50%/100%/150%, Entreprise dégradée 150%, Procédure prudentielle 150%). Laissez « Standard » ou vide si aucun traitement particulier ne s'applique.</t>
         </is>
       </c>
     </row>
@@ -3285,7 +3369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT5"/>
+  <dimension ref="A1:AD7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3313,27 +3397,11 @@
     <col width="16" customWidth="1" min="23" max="23"/>
     <col width="17" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="29" customWidth="1" min="26" max="26"/>
-    <col width="36" customWidth="1" min="27" max="27"/>
-    <col width="24" customWidth="1" min="28" max="28"/>
-    <col width="22" customWidth="1" min="29" max="29"/>
-    <col width="35" customWidth="1" min="30" max="30"/>
-    <col width="38" customWidth="1" min="31" max="31"/>
-    <col width="25" customWidth="1" min="32" max="32"/>
-    <col width="22" customWidth="1" min="33" max="33"/>
-    <col width="32" customWidth="1" min="34" max="34"/>
-    <col width="31" customWidth="1" min="35" max="35"/>
-    <col width="28" customWidth="1" min="36" max="36"/>
-    <col width="20" customWidth="1" min="37" max="37"/>
-    <col width="38" customWidth="1" min="38" max="38"/>
-    <col width="35" customWidth="1" min="39" max="39"/>
-    <col width="34" customWidth="1" min="40" max="40"/>
-    <col width="37" customWidth="1" min="41" max="41"/>
-    <col width="32" customWidth="1" min="42" max="42"/>
-    <col width="30" customWidth="1" min="43" max="43"/>
-    <col width="38" customWidth="1" min="44" max="44"/>
-    <col width="37" customWidth="1" min="45" max="45"/>
-    <col width="38" customWidth="1" min="46" max="46"/>
+    <col width="32" customWidth="1" min="26" max="26"/>
+    <col width="29" customWidth="1" min="27" max="27"/>
+    <col width="22" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="37" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3464,476 +3532,848 @@
       </c>
       <c r="Z1" s="5" t="inlineStr">
         <is>
+          <t>Regime_prudentiel_specifique</t>
+        </is>
+      </c>
+      <c r="AA1" s="5" t="inlineStr">
+        <is>
           <t>Cas_particulier_souverain</t>
         </is>
       </c>
-      <c r="AA1" s="6" t="inlineStr">
-        <is>
-          <t>Souverain_ponderation_pref_nulle</t>
-        </is>
-      </c>
-      <c r="AB1" s="6" t="inlineStr">
-        <is>
-          <t>Souverain_OCE_etabli</t>
+      <c r="AB1" s="5" t="inlineStr">
+        <is>
+          <t>Souverain_note_OCE</t>
         </is>
       </c>
       <c r="AC1" s="5" t="inlineStr">
         <is>
-          <t>Souverain_note_OCE</t>
-        </is>
-      </c>
-      <c r="AD1" s="6" t="inlineStr">
-        <is>
-          <t>Organisme_public_cas_UEMOA_FCFA</t>
-        </is>
-      </c>
-      <c r="AE1" s="6" t="inlineStr">
-        <is>
-          <t>Organisme_public_activite_non_publique</t>
-        </is>
-      </c>
-      <c r="AF1" s="6" t="inlineStr">
-        <is>
-          <t>BMD_cas_haute_qualite</t>
-        </is>
-      </c>
-      <c r="AG1" s="6" t="inlineStr">
-        <is>
-          <t>BMD_cas_UEMOA_FCFA</t>
-        </is>
-      </c>
-      <c r="AH1" s="6" t="inlineStr">
-        <is>
-          <t>BMD_criteres_UEMOA_respectes</t>
-        </is>
-      </c>
-      <c r="AI1" s="6" t="inlineStr">
-        <is>
-          <t>BMD_institution_listee_FCFA</t>
-        </is>
-      </c>
-      <c r="AJ1" s="5" t="inlineStr">
-        <is>
-          <t>Cas_institution_bancaire</t>
-        </is>
-      </c>
-      <c r="AK1" s="5" t="inlineStr">
-        <is>
           <t>Type_autre_actif</t>
         </is>
       </c>
-      <c r="AL1" s="6" t="inlineStr">
-        <is>
-          <t>Clientele_detail_criteres_respectes</t>
-        </is>
-      </c>
-      <c r="AM1" s="6" t="inlineStr">
-        <is>
-          <t>Immobilier_residentiel_eligible</t>
-        </is>
-      </c>
-      <c r="AN1" s="6" t="inlineStr">
-        <is>
-          <t>Immobilier_commercial_eligible</t>
-        </is>
-      </c>
-      <c r="AO1" s="5" t="inlineStr">
+      <c r="AD1" s="5" t="inlineStr">
         <is>
           <t>Ponderation_initiale_avant_defaut</t>
         </is>
       </c>
-      <c r="AP1" s="6" t="inlineStr">
-        <is>
-          <t>Defaut_pret_immo_residentiel</t>
-        </is>
-      </c>
-      <c r="AQ1" s="6" t="inlineStr">
-        <is>
-          <t>Defaut_provision_min_20pct</t>
-        </is>
-      </c>
-      <c r="AR1" s="6" t="inlineStr">
-        <is>
-          <t>Entreprise_depasse_seuil_degradation_BCEAO</t>
-        </is>
-      </c>
-      <c r="AS1" s="6" t="inlineStr">
-        <is>
-          <t>Entreprise_procedure_prudentielle</t>
-        </is>
-      </c>
-      <c r="AT1" s="6" t="inlineStr">
-        <is>
-          <t>Entreprise_investissement_hors_loi_bancaire</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>EXP-EX-001</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>État XYZ</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Trésor Public de Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Côte d'Ivoire</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Souverains</t>
         </is>
       </c>
-      <c r="H2" s="7" t="n">
+      <c r="H2" s="6" t="n">
         <v>500000000</v>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>XOF</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>Aucune</t>
         </is>
       </c>
-      <c r="K2" s="7" t="n"/>
-      <c r="L2" s="7" t="n"/>
-      <c r="M2" s="7" t="n"/>
-      <c r="N2" s="7" t="n"/>
-      <c r="O2" s="7" t="n"/>
-      <c r="P2" s="7" t="n"/>
-      <c r="Q2" s="7" t="n"/>
-      <c r="R2" s="7" t="n"/>
-      <c r="S2" s="7" t="n"/>
-      <c r="T2" s="7" t="n"/>
-      <c r="U2" s="7" t="n"/>
-      <c r="V2" s="7" t="n"/>
-      <c r="W2" s="7" t="n"/>
-      <c r="X2" s="7" t="n"/>
-      <c r="Y2" s="7" t="n"/>
-      <c r="Z2" s="7" t="n"/>
-      <c r="AA2" s="7" t="n"/>
-      <c r="AB2" s="7" t="n"/>
-      <c r="AC2" s="7" t="n"/>
-      <c r="AD2" s="7" t="n"/>
-      <c r="AE2" s="7" t="n"/>
-      <c r="AF2" s="7" t="n"/>
-      <c r="AG2" s="7" t="n"/>
-      <c r="AH2" s="7" t="n"/>
-      <c r="AI2" s="7" t="n"/>
-      <c r="AJ2" s="7" t="n"/>
-      <c r="AK2" s="7" t="n"/>
-      <c r="AL2" s="7" t="n"/>
-      <c r="AM2" s="7" t="n"/>
-      <c r="AN2" s="7" t="n"/>
-      <c r="AO2" s="7" t="n"/>
-      <c r="AP2" s="7" t="n"/>
-      <c r="AQ2" s="7" t="n"/>
-      <c r="AR2" s="7" t="n"/>
-      <c r="AS2" s="7" t="n"/>
-      <c r="AT2" s="7" t="n"/>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>CR-CI-0001</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Administration publique</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="P2" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="Q2" s="6" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>2029-01-15</t>
+        </is>
+      </c>
+      <c r="S2" s="6" t="n">
+        <v>500000000</v>
+      </c>
+      <c r="T2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t>Risque faible</t>
+        </is>
+      </c>
+      <c r="V2" s="6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="W2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="6" t="inlineStr">
+        <is>
+          <t>Bons du Trésor UEMOA — éligible refinancement BCEAO</t>
+        </is>
+      </c>
+      <c r="Z2" s="6" t="inlineStr">
+        <is>
+          <t>Souverain UEMOA en FCFA (pondération 0 %)</t>
+        </is>
+      </c>
+      <c r="AA2" s="6" t="inlineStr">
+        <is>
+          <t>Traitement préférentiel UEMOA (0%)</t>
+        </is>
+      </c>
+      <c r="AB2" s="6" t="n"/>
+      <c r="AC2" s="6" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AD2" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>EXP-EX-002</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Société ABC SA</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Société Industrielle Ivoirienne SA</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Côte d'Ivoire</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Entreprises</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>XOF</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>CRM financee</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>CR-CI-0114</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>Industrie manufacturiere</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>Groupe Industriel Ivoirien</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>CR-CI-0100</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>Controle de droit</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="Q3" s="7" t="inlineStr">
+        <is>
+          <t>2023-05-10</t>
+        </is>
+      </c>
+      <c r="R3" s="7" t="inlineStr">
+        <is>
+          <t>2027-05-10</t>
+        </is>
+      </c>
+      <c r="S3" s="7" t="n">
+        <v>180000000</v>
+      </c>
+      <c r="T3" s="7" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="U3" s="7" t="inlineStr">
+        <is>
+          <t>Risque moyen</t>
+        </is>
+      </c>
+      <c r="V3" s="7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="W3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="7" t="inlineStr">
+        <is>
+          <t>Ligne de crédit adossée à garantie espèces nantie</t>
+        </is>
+      </c>
+      <c r="Z3" s="7" t="inlineStr">
+        <is>
+          <t>Standard (aucun traitement particulier)</t>
+        </is>
+      </c>
+      <c r="AA3" s="7" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AB3" s="7" t="n"/>
+      <c r="AC3" s="7" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AD3" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>EXP-EX-003</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Particulier — M. Amadou Diallo</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Non noté</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Sénégal</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Clientèle de détail</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>XOF</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>CRM non financee</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>CR-SN-0207</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Menages</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="P4" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="Q4" s="6" t="inlineStr">
+        <is>
+          <t>2024-03-01</t>
+        </is>
+      </c>
+      <c r="R4" s="6" t="inlineStr">
+        <is>
+          <t>2028-03-01</t>
+        </is>
+      </c>
+      <c r="S4" s="6" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="T4" s="6" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="U4" s="6" t="inlineStr">
+        <is>
+          <t>Risque moyen</t>
+        </is>
+      </c>
+      <c r="V4" s="6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="W4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="6" t="inlineStr">
+        <is>
+          <t>Crédit équipement couvert par caution souveraine</t>
+        </is>
+      </c>
+      <c r="Z4" s="6" t="inlineStr">
+        <is>
+          <t>Clientèle de détail - Critères d'éligibilité respectés (pondération 75 %)</t>
+        </is>
+      </c>
+      <c r="AA4" s="6" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AB4" s="6" t="n"/>
+      <c r="AC4" s="6" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AD4" s="6" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>EXP-EX-004</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Particulier — Mme Fatou Traoré</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Non noté</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Mali</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Immobilier résidentiel</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>XOF</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="K5" s="7" t="inlineStr">
+        <is>
+          <t>CR-ML-0318</t>
+        </is>
+      </c>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Menages</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="N5" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="P5" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="Q5" s="7" t="inlineStr">
+        <is>
+          <t>2022-09-15</t>
+        </is>
+      </c>
+      <c r="R5" s="7" t="inlineStr">
+        <is>
+          <t>2037-09-15</t>
+        </is>
+      </c>
+      <c r="S5" s="7" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="T5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="7" t="inlineStr">
+        <is>
+          <t>Risque faible</t>
+        </is>
+      </c>
+      <c r="V5" s="7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="W5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="7" t="inlineStr">
+        <is>
+          <t>Crédit acquisition logement avec hypothèque 1er rang</t>
+        </is>
+      </c>
+      <c r="Z5" s="7" t="inlineStr">
+        <is>
+          <t>Immobilier résidentiel - Prêt éligible avec hypothèque 1er rang (pondération 35 %)</t>
+        </is>
+      </c>
+      <c r="AA5" s="7" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AB5" s="7" t="n"/>
+      <c r="AC5" s="7" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AD5" s="7" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>EXP-EX-005</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Entreprise Sahel Négoce SARL</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>&lt; B-</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Burkina Faso</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>BB</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Sénégal</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Entreprises</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="n">
-        <v>150000000</v>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Créances en souffrance</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>XOF</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>CRM financee</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="n"/>
-      <c r="L3" s="8" t="n"/>
-      <c r="M3" s="8" t="n"/>
-      <c r="N3" s="8" t="n"/>
-      <c r="O3" s="8" t="n"/>
-      <c r="P3" s="8" t="n"/>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>2024-01-10</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>2027-01-10</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="n">
-        <v>160000000</v>
-      </c>
-      <c r="T3" s="8" t="n"/>
-      <c r="U3" s="8" t="n"/>
-      <c r="V3" s="8" t="n"/>
-      <c r="W3" s="8" t="n"/>
-      <c r="X3" s="8" t="n"/>
-      <c r="Y3" s="8" t="n"/>
-      <c r="Z3" s="8" t="n"/>
-      <c r="AA3" s="8" t="n"/>
-      <c r="AB3" s="8" t="n"/>
-      <c r="AC3" s="8" t="n"/>
-      <c r="AD3" s="8" t="n"/>
-      <c r="AE3" s="8" t="n"/>
-      <c r="AF3" s="8" t="n"/>
-      <c r="AG3" s="8" t="n"/>
-      <c r="AH3" s="8" t="n"/>
-      <c r="AI3" s="8" t="n"/>
-      <c r="AJ3" s="8" t="n"/>
-      <c r="AK3" s="8" t="n"/>
-      <c r="AL3" s="8" t="n"/>
-      <c r="AM3" s="8" t="n"/>
-      <c r="AN3" s="8" t="n"/>
-      <c r="AO3" s="8" t="n"/>
-      <c r="AP3" s="8" t="n"/>
-      <c r="AQ3" s="8" t="n"/>
-      <c r="AR3" s="8" t="n"/>
-      <c r="AS3" s="8" t="n"/>
-      <c r="AT3" s="8" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>CR-BF-0422</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Commerce de gros et de detail</t>
+        </is>
+      </c>
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>Groupe Industriel Ivoirien</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>CR-CI-0100</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>Dependance economique</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="Q6" s="6" t="inlineStr">
+        <is>
+          <t>2023-02-01</t>
+        </is>
+      </c>
+      <c r="R6" s="6" t="inlineStr">
+        <is>
+          <t>2025-02-01</t>
+        </is>
+      </c>
+      <c r="S6" s="6" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="T6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t>Risque très élevé</t>
+        </is>
+      </c>
+      <c r="V6" s="6" t="inlineStr">
+        <is>
+          <t>Contentieux</t>
+        </is>
+      </c>
+      <c r="W6" s="6" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="X6" s="6" t="n">
+        <v>125</v>
+      </c>
+      <c r="Y6" s="6" t="inlineStr">
+        <is>
+          <t>Dossier contentieux avec provisionnement à 32%</t>
+        </is>
+      </c>
+      <c r="Z6" s="6" t="inlineStr">
+        <is>
+          <t>Défaut - Autre créance en souffrance (Provisions &gt;= 20%) — pondération 100 %</t>
+        </is>
+      </c>
+      <c r="AA6" s="6" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AB6" s="6" t="n"/>
+      <c r="AC6" s="6" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AD6" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>EXP-EX-003</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Particulier — M. Koffi</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>EXP-EX-006</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Valeurs en caisse et avoirs BCEAO</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Non noté</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Côte d'Ivoire</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Clientèle de détail</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="n">
-        <v>8000000</v>
-      </c>
-      <c r="I4" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Autres actifs</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>XOF</t>
         </is>
       </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>CRM non financee</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
-      <c r="M4" s="7" t="n"/>
-      <c r="N4" s="7" t="n"/>
-      <c r="O4" s="7" t="n"/>
-      <c r="P4" s="7" t="n"/>
-      <c r="Q4" s="7" t="n"/>
-      <c r="R4" s="7" t="n"/>
-      <c r="S4" s="7" t="n"/>
-      <c r="T4" s="7" t="n">
-        <v>2000000</v>
-      </c>
-      <c r="U4" s="7" t="inlineStr">
-        <is>
-          <t>Risque moyen</t>
-        </is>
-      </c>
-      <c r="V4" s="7" t="n"/>
-      <c r="W4" s="7" t="n"/>
-      <c r="X4" s="7" t="n"/>
-      <c r="Y4" s="7" t="n"/>
-      <c r="Z4" s="7" t="n"/>
-      <c r="AA4" s="7" t="n"/>
-      <c r="AB4" s="7" t="n"/>
-      <c r="AC4" s="7" t="n"/>
-      <c r="AD4" s="7" t="n"/>
-      <c r="AE4" s="7" t="n"/>
-      <c r="AF4" s="7" t="n"/>
-      <c r="AG4" s="7" t="n"/>
-      <c r="AH4" s="7" t="n"/>
-      <c r="AI4" s="7" t="n"/>
-      <c r="AJ4" s="7" t="n"/>
-      <c r="AK4" s="7" t="n"/>
-      <c r="AL4" s="7" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="AM4" s="7" t="n"/>
-      <c r="AN4" s="7" t="n"/>
-      <c r="AO4" s="7" t="n"/>
-      <c r="AP4" s="7" t="n"/>
-      <c r="AQ4" s="7" t="n"/>
-      <c r="AR4" s="7" t="n"/>
-      <c r="AS4" s="7" t="n"/>
-      <c r="AT4" s="7" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Aucune</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>CR-CI-0500</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Activites financieres et d'assurance</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>Néant</t>
+        </is>
+      </c>
+      <c r="Q7" s="7" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>EXP-EX-004</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Banque Régionale XYZ</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Bénin</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Institutions financières</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="n">
-        <v>75000000</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>XOF</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>Aucune</t>
-        </is>
-      </c>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-      <c r="M5" s="8" t="n"/>
-      <c r="N5" s="8" t="n"/>
-      <c r="O5" s="8" t="n"/>
-      <c r="P5" s="8" t="n"/>
-      <c r="Q5" s="8" t="n"/>
-      <c r="R5" s="8" t="n"/>
-      <c r="S5" s="8" t="n"/>
-      <c r="T5" s="8" t="n"/>
-      <c r="U5" s="8" t="n"/>
-      <c r="V5" s="8" t="n"/>
-      <c r="W5" s="8" t="n"/>
-      <c r="X5" s="8" t="n"/>
-      <c r="Y5" s="8" t="n"/>
-      <c r="Z5" s="8" t="n"/>
-      <c r="AA5" s="8" t="n"/>
-      <c r="AB5" s="8" t="n"/>
-      <c r="AC5" s="8" t="n"/>
-      <c r="AD5" s="8" t="n"/>
-      <c r="AE5" s="8" t="n"/>
-      <c r="AF5" s="8" t="n"/>
-      <c r="AG5" s="8" t="n"/>
-      <c r="AH5" s="8" t="n"/>
-      <c r="AI5" s="8" t="n"/>
-      <c r="AJ5" s="8" t="n"/>
-      <c r="AK5" s="8" t="n"/>
-      <c r="AL5" s="8" t="n"/>
-      <c r="AM5" s="8" t="n"/>
-      <c r="AN5" s="8" t="n"/>
-      <c r="AO5" s="8" t="n"/>
-      <c r="AP5" s="8" t="n"/>
-      <c r="AQ5" s="8" t="n"/>
-      <c r="AR5" s="8" t="n"/>
-      <c r="AS5" s="8" t="n"/>
-      <c r="AT5" s="8" t="n"/>
+      <c r="R7" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="S7" s="7" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="T7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="7" t="inlineStr">
+        <is>
+          <t>Risque faible</t>
+        </is>
+      </c>
+      <c r="V7" s="7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="W7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="7" t="inlineStr">
+        <is>
+          <t>Billets et monnaies en caisse</t>
+        </is>
+      </c>
+      <c r="Z7" s="7" t="inlineStr">
+        <is>
+          <t>Standard (aucun traitement particulier)</t>
+        </is>
+      </c>
+      <c r="AA7" s="7" t="inlineStr">
+        <is>
+          <t>(Sans objet pour cette catégorie)</t>
+        </is>
+      </c>
+      <c r="AB7" s="7" t="n"/>
+      <c r="AC7" s="7" t="inlineStr">
+        <is>
+          <t>Billets et monnaies en caisse (0 %)</t>
+        </is>
+      </c>
+      <c r="AD7" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="23">
+  <dataValidations count="15">
     <dataValidation sqref="D2:D2001 F2:F2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
       <formula1>'Listes (validation)'!$E$2:$E$19</formula1>
     </dataValidation>
@@ -3950,13 +4390,13 @@
       <formula1>'Listes (validation)'!$C$2:$C$4</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$O$2:$O$22</formula1>
+      <formula1>'Listes (validation)'!$T$2:$T$22</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$M$2:$M$4</formula1>
+      <formula1>'Listes (validation)'!$R$2:$R$4</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$N$2:$N$9</formula1>
+      <formula1>'Listes (validation)'!$S$2:$S$9</formula1>
     </dataValidation>
     <dataValidation sqref="U2:U2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
       <formula1>'Listes (validation)'!$G$2:$G$6</formula1>
@@ -3965,43 +4405,19 @@
       <formula1>'Listes (validation)'!$H$2:$H$6</formula1>
     </dataValidation>
     <dataValidation sqref="Z2:Z2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Souverains","ListeCascade2","ListeCascade1"))</formula1>
+      <formula1>'Listes (validation)'!$I$2:$I$20</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA2001 AB2:AB2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Souverains","ListeCascade3","ListeCascade1"))</formula1>
+    <dataValidation sqref="AA2:AA2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
+      <formula1>'Listes (validation)'!$J$2:$J$13</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB2:AB2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
+      <formula1>'Listes (validation)'!$K$2:$K$9</formula1>
     </dataValidation>
     <dataValidation sqref="AC2:AC2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Souverains","ListeCascade4","ListeCascade1"))</formula1>
+      <formula1>'Listes (validation)'!$Q$2:$Q$14</formula1>
     </dataValidation>
-    <dataValidation sqref="AD2:AD2001 AE2:AE2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Organismes pub. hors Adm c","ListeCascade3","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AF2:AF2001 AG2:AG2001 AH2:AH2001 AI2:AI2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Expositions sur les BMD","ListeCascade3","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AJ2:AJ2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Institutions financières","ListeCascade5","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AK2:AK2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Autres actifs","ListeCascade6","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AL2:AL2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Clientèle de détail","ListeCascade3","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AM2:AM2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Prêts garantis par l'immo R","ListeCascade3","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AN2:AN2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Prêts garantis par l'immo C","ListeCascade3","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AO2:AO2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Créances en souffrance","ListeCascade7","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AP2:AP2001 AQ2:AQ2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF($G2="Créances en souffrance","ListeCascade3","ListeCascade1"))</formula1>
-    </dataValidation>
-    <dataValidation sqref="AR2:AR2001 AS2:AS2001 AT2:AT2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>INDIRECT(IF(OR($G2="Entreprises",$G2="Clientèle de détail",$G2="Prêts garantis par l'immo C"),"ListeCascade3","ListeCascade1"))</formula1>
+    <dataValidation sqref="AD2:AD2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
+      <formula1>'Listes (validation)'!$U$2:$U$8</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4065,44 +4481,44 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>EXP-EX-003</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Fonds de Garantie XYZ</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Souverains</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Côte d'Ivoire</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="G2" s="6" t="n">
         <v>1500000</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C2:C2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$Q$2:$Q$8</formula1>
+      <formula1>'Listes (validation)'!$V$2:$V$8</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D2001 F2:F2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
       <formula1>'Listes (validation)'!$E$2:$E$19</formula1>
@@ -4178,7 +4594,7 @@
           <t>Type_Collatéral</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="8" t="inlineStr">
         <is>
           <t>Obligation_convertible_indice_principal</t>
         </is>
@@ -4190,61 +4606,61 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>EXP-EX-002</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
+      <c r="B2" s="6" t="n">
         <v>50000000</v>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>emprunteur souverain</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>AAA</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Garantie espèces</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>&lt;=1 an</t>
         </is>
       </c>
-      <c r="G2" s="7" t="n"/>
-      <c r="H2" s="7" t="n"/>
-      <c r="I2" s="7" t="n"/>
-      <c r="J2" s="7" t="n"/>
+      <c r="G2" s="6" t="n"/>
+      <c r="H2" s="6" t="n"/>
+      <c r="I2" s="6" t="n"/>
+      <c r="J2" s="6" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="7">
     <dataValidation sqref="C2:C2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$R$2:$R$3</formula1>
+      <formula1>'Listes (validation)'!$W$2:$W$3</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$S$2:$S$16</formula1>
+      <formula1>'Listes (validation)'!$X$2:$X$16</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$T$2:$T$6</formula1>
+      <formula1>'Listes (validation)'!$Y$2:$Y$6</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
       <formula1>'Listes (validation)'!$D$2:$D$4</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$U$2:$U$16</formula1>
+      <formula1>'Listes (validation)'!$Z$2:$Z$16</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
       <formula1>'Listes (validation)'!$A$2:$A$3</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez une valeur dans la liste déroulante pour que le calcul prudentiel s'applique correctement à cette ligne." type="list">
-      <formula1>'Listes (validation)'!$V$2:$V$13</formula1>
+      <formula1>'Listes (validation)'!$AA$2:$AA$13</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4258,7 +4674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B169"/>
+  <dimension ref="A1:B213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4371,7 +4787,7 @@
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>Type_CRM</t>
+          <t>Régime prudentiel spécifique (BCEAO)</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr"/>
@@ -4379,7 +4795,7 @@
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>Standard (aucun traitement particulier)</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr"/>
@@ -4387,7 +4803,7 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>CRM financee</t>
+          <t>Souverain UEMOA en FCFA (pondération 0 %)</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr"/>
@@ -4395,23 +4811,31 @@
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>CRM non financee</t>
+          <t>Organisme public UEMOA en FCFA (pondération 20 %)</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr"/>
     </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Organisme public - Activité commerciale (traité comme entreprise)</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr"/>
+    </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>Niveau de risque HB</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr"/>
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>BMD liste officielle BCEAO (BIRD, BAD, BOAD... pondération 0 %)</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>Risque faible</t>
+          <t>BMD haute qualité / soutien fort (pondération 0 %)</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr"/>
@@ -4419,7 +4843,7 @@
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
         <is>
-          <t>Risque mineur</t>
+          <t>BMD UEMOA en FCFA (pondération 20 %)</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr"/>
@@ -4427,7 +4851,7 @@
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Risque moyen</t>
+          <t>Banque - Établissement de crédit agréé UEMOA</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr"/>
@@ -4435,7 +4859,7 @@
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>Risque élevé</t>
+          <t>Banque - Faible qualité prudentielle</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr"/>
@@ -4443,23 +4867,31 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Risque très élevé</t>
+          <t>Clientèle de détail - Critères d'éligibilité respectés (pondération 75 %)</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr"/>
     </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Immobilier résidentiel - Prêt éligible avec hypothèque 1er rang (pondération 35 %)</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr"/>
+    </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>Statut (gestion)</t>
-        </is>
-      </c>
-      <c r="B28" s="11" t="inlineStr"/>
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Immobilier commercial - Prêt éligible (pondération 50 %)</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Défaut - Prêt immobilier résidentiel (Provisions &gt;= 20%) — pondération 50 %</t>
         </is>
       </c>
       <c r="B29" s="13" t="inlineStr"/>
@@ -4467,7 +4899,7 @@
     <row r="30">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>En recouvrement</t>
+          <t>Défaut - Prêt immobilier résidentiel (Provisions &lt; 20%) — pondération 100 %</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr"/>
@@ -4475,7 +4907,7 @@
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>Restructurée</t>
+          <t>Défaut - Autre créance en souffrance (Provisions &gt;= 20%) — pondération 100 %</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr"/>
@@ -4483,7 +4915,7 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Contentieux</t>
+          <t>Défaut - Autre créance en souffrance (Provisions &lt; 20%) — pondération 150 %</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr"/>
@@ -4491,39 +4923,39 @@
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>Clôturée</t>
+          <t>Entreprise - Portefeuille dégradé (seuil BCEAO dépassé -&gt; pondération 150 %)</t>
         </is>
       </c>
       <c r="B33" s="13" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>Entreprise - Procédure prudentielle (pondération 150 %)</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr"/>
+    </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Catégorie du garant (CRM non financée)</t>
-        </is>
-      </c>
-      <c r="B35" s="11" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
-        <is>
-          <t>Souverains</t>
-        </is>
-      </c>
-      <c r="B36" s="13" t="inlineStr"/>
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>Entreprise d'investissement non soumise à la loi bancaire (pondération 100 %)</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>Organismes pub. hors Adm c</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="inlineStr"/>
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>Type_CRM</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>Expositions sur les BMD</t>
+          <t>Aucune</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr"/>
@@ -4531,7 +4963,7 @@
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>Institutions financières</t>
+          <t>CRM financee</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr"/>
@@ -4539,39 +4971,39 @@
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>Entreprises</t>
+          <t>CRM non financee</t>
         </is>
       </c>
       <c r="B40" s="13" t="inlineStr"/>
     </row>
-    <row r="41">
-      <c r="A41" s="14" t="inlineStr">
-        <is>
-          <t>Clientèle de détail</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="inlineStr"/>
-    </row>
     <row r="42">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t>Autres actifs</t>
-        </is>
-      </c>
-      <c r="B42" s="13" t="inlineStr"/>
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>Niveau de risque HB</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
+        <is>
+          <t>Risque faible</t>
+        </is>
+      </c>
+      <c r="B43" s="13" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>Notation (contrepartie / pays / garant)</t>
-        </is>
-      </c>
-      <c r="B44" s="11" t="inlineStr"/>
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>Risque mineur</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>AAA</t>
+          <t>Risque moyen</t>
         </is>
       </c>
       <c r="B45" s="13" t="inlineStr"/>
@@ -4579,7 +5011,7 @@
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t>AA+</t>
+          <t>Risque élevé</t>
         </is>
       </c>
       <c r="B46" s="13" t="inlineStr"/>
@@ -4587,31 +5019,23 @@
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>Risque très élevé</t>
         </is>
       </c>
       <c r="B47" s="13" t="inlineStr"/>
     </row>
-    <row r="48">
-      <c r="A48" s="12" t="inlineStr">
-        <is>
-          <t>AA-</t>
-        </is>
-      </c>
-      <c r="B48" s="13" t="inlineStr"/>
-    </row>
     <row r="49">
-      <c r="A49" s="14" t="inlineStr">
-        <is>
-          <t>A+</t>
-        </is>
-      </c>
-      <c r="B49" s="13" t="inlineStr"/>
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Statut (gestion)</t>
+        </is>
+      </c>
+      <c r="B49" s="11" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="B50" s="13" t="inlineStr"/>
@@ -4619,7 +5043,7 @@
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>A-</t>
+          <t>En recouvrement</t>
         </is>
       </c>
       <c r="B51" s="13" t="inlineStr"/>
@@ -4627,7 +5051,7 @@
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
         <is>
-          <t>BBB+</t>
+          <t>Restructurée</t>
         </is>
       </c>
       <c r="B52" s="13" t="inlineStr"/>
@@ -4635,7 +5059,7 @@
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>BBB</t>
+          <t>Contentieux</t>
         </is>
       </c>
       <c r="B53" s="13" t="inlineStr"/>
@@ -4643,31 +5067,23 @@
     <row r="54">
       <c r="A54" s="12" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>Clôturée</t>
         </is>
       </c>
       <c r="B54" s="13" t="inlineStr"/>
     </row>
-    <row r="55">
-      <c r="A55" s="14" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-      <c r="B55" s="13" t="inlineStr"/>
-    </row>
     <row r="56">
-      <c r="A56" s="12" t="inlineStr">
-        <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="B56" s="13" t="inlineStr"/>
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>Catégorie du garant (CRM non financée)</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>Souverains</t>
         </is>
       </c>
       <c r="B57" s="13" t="inlineStr"/>
@@ -4675,7 +5091,7 @@
     <row r="58">
       <c r="A58" s="12" t="inlineStr">
         <is>
-          <t>B+</t>
+          <t>Organismes pub. hors Adm c</t>
         </is>
       </c>
       <c r="B58" s="13" t="inlineStr"/>
@@ -4683,7 +5099,7 @@
     <row r="59">
       <c r="A59" s="14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>Expositions sur les BMD</t>
         </is>
       </c>
       <c r="B59" s="13" t="inlineStr"/>
@@ -4691,7 +5107,7 @@
     <row r="60">
       <c r="A60" s="12" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>Institutions financières</t>
         </is>
       </c>
       <c r="B60" s="13" t="inlineStr"/>
@@ -4699,7 +5115,7 @@
     <row r="61">
       <c r="A61" s="14" t="inlineStr">
         <is>
-          <t>&lt; B-</t>
+          <t>Entreprises</t>
         </is>
       </c>
       <c r="B61" s="13" t="inlineStr"/>
@@ -4707,31 +5123,31 @@
     <row r="62">
       <c r="A62" s="12" t="inlineStr">
         <is>
-          <t>Non noté</t>
+          <t>Clientèle de détail</t>
         </is>
       </c>
       <c r="B62" s="13" t="inlineStr"/>
     </row>
-    <row r="64">
-      <c r="A64" s="10" t="inlineStr">
-        <is>
-          <t>Notation (collatéral CRM financée)</t>
-        </is>
-      </c>
-      <c r="B64" s="11" t="inlineStr"/>
+    <row r="63">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>Autres actifs</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="14" t="inlineStr">
-        <is>
-          <t>AAA</t>
-        </is>
-      </c>
-      <c r="B65" s="13" t="inlineStr"/>
+      <c r="A65" s="10" t="inlineStr">
+        <is>
+          <t>Notation (contrepartie / pays / garant)</t>
+        </is>
+      </c>
+      <c r="B65" s="11" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
         <is>
-          <t>AA+</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="B66" s="13" t="inlineStr"/>
@@ -4739,7 +5155,7 @@
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>AA</t>
+          <t>AA+</t>
         </is>
       </c>
       <c r="B67" s="13" t="inlineStr"/>
@@ -4747,7 +5163,7 @@
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
         <is>
-          <t>AA-</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="B68" s="13" t="inlineStr"/>
@@ -4755,7 +5171,7 @@
     <row r="69">
       <c r="A69" s="14" t="inlineStr">
         <is>
-          <t>A+</t>
+          <t>AA-</t>
         </is>
       </c>
       <c r="B69" s="13" t="inlineStr"/>
@@ -4763,7 +5179,7 @@
     <row r="70">
       <c r="A70" s="12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="B70" s="13" t="inlineStr"/>
@@ -4771,7 +5187,7 @@
     <row r="71">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>A-</t>
+          <t>A</t>
         </is>
       </c>
       <c r="B71" s="13" t="inlineStr"/>
@@ -4779,7 +5195,7 @@
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
         <is>
-          <t>BBB+</t>
+          <t>A-</t>
         </is>
       </c>
       <c r="B72" s="13" t="inlineStr"/>
@@ -4787,7 +5203,7 @@
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
         <is>
-          <t>BBB</t>
+          <t>BBB+</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr"/>
@@ -4795,7 +5211,7 @@
     <row r="74">
       <c r="A74" s="12" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>BBB</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr"/>
@@ -4803,7 +5219,7 @@
     <row r="75">
       <c r="A75" s="14" t="inlineStr">
         <is>
-          <t>BB+</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="B75" s="13" t="inlineStr"/>
@@ -4811,7 +5227,7 @@
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="B76" s="13" t="inlineStr"/>
@@ -4819,7 +5235,7 @@
     <row r="77">
       <c r="A77" s="14" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B77" s="13" t="inlineStr"/>
@@ -4827,7 +5243,7 @@
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
-          <t>&lt; B-</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="B78" s="13" t="inlineStr"/>
@@ -4835,23 +5251,31 @@
     <row r="79">
       <c r="A79" s="14" t="inlineStr">
         <is>
-          <t>Non noté</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="B79" s="13" t="inlineStr"/>
     </row>
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="inlineStr"/>
+    </row>
     <row r="81">
-      <c r="A81" s="10" t="inlineStr">
-        <is>
-          <t>Type_emetteur (CRM financée)</t>
-        </is>
-      </c>
-      <c r="B81" s="11" t="inlineStr"/>
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="B81" s="13" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t>emprunteur souverain</t>
+          <t>&lt; B-</t>
         </is>
       </c>
       <c r="B82" s="13" t="inlineStr"/>
@@ -4859,7 +5283,7 @@
     <row r="83">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>autre émetteur</t>
+          <t>Non noté</t>
         </is>
       </c>
       <c r="B83" s="13" t="inlineStr"/>
@@ -4867,7 +5291,7 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>Maturite (CRM financée)</t>
+          <t>Notation (collatéral CRM financée)</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr"/>
@@ -4875,7 +5299,7 @@
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t>&lt;=1 an</t>
+          <t>AAA</t>
         </is>
       </c>
       <c r="B86" s="13" t="inlineStr"/>
@@ -4883,7 +5307,7 @@
     <row r="87">
       <c r="A87" s="14" t="inlineStr">
         <is>
-          <t>1-3 ans</t>
+          <t>AA+</t>
         </is>
       </c>
       <c r="B87" s="13" t="inlineStr"/>
@@ -4891,7 +5315,7 @@
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t>3-5 ans</t>
+          <t>AA</t>
         </is>
       </c>
       <c r="B88" s="13" t="inlineStr"/>
@@ -4899,7 +5323,7 @@
     <row r="89">
       <c r="A89" s="14" t="inlineStr">
         <is>
-          <t>5-10 ans</t>
+          <t>AA-</t>
         </is>
       </c>
       <c r="B89" s="13" t="inlineStr"/>
@@ -4907,23 +5331,31 @@
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t>&gt;10 ans</t>
+          <t>A+</t>
         </is>
       </c>
       <c r="B90" s="13" t="inlineStr"/>
     </row>
+    <row r="91">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B91" s="13" t="inlineStr"/>
+    </row>
     <row r="92">
-      <c r="A92" s="10" t="inlineStr">
-        <is>
-          <t>Type_Collatéral (CRM financée)</t>
-        </is>
-      </c>
-      <c r="B92" s="11" t="inlineStr"/>
+      <c r="A92" s="12" t="inlineStr">
+        <is>
+          <t>A-</t>
+        </is>
+      </c>
+      <c r="B92" s="13" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="14" t="inlineStr">
         <is>
-          <t>Liquidités dans la même devise</t>
+          <t>BBB+</t>
         </is>
       </c>
       <c r="B93" s="13" t="inlineStr"/>
@@ -4931,7 +5363,7 @@
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
         <is>
-          <t>Liquidités dans une devise différente</t>
+          <t>BBB</t>
         </is>
       </c>
       <c r="B94" s="13" t="inlineStr"/>
@@ -4939,7 +5371,7 @@
     <row r="95">
       <c r="A95" s="14" t="inlineStr">
         <is>
-          <t>Or</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="B95" s="13" t="inlineStr"/>
@@ -4947,7 +5379,7 @@
     <row r="96">
       <c r="A96" s="12" t="inlineStr">
         <is>
-          <t>Titre de dette souverain</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="B96" s="13" t="inlineStr"/>
@@ -4955,7 +5387,7 @@
     <row r="97">
       <c r="A97" s="14" t="inlineStr">
         <is>
-          <t>Titre non noté émis par un État de l UMOA</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="B97" s="13" t="inlineStr"/>
@@ -4963,7 +5395,7 @@
     <row r="98">
       <c r="A98" s="12" t="inlineStr">
         <is>
-          <t>Titre de dette émis par un autre émetteur</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="B98" s="13" t="inlineStr"/>
@@ -4971,7 +5403,7 @@
     <row r="99">
       <c r="A99" s="14" t="inlineStr">
         <is>
-          <t>Titre garanti par un agent agréé par la BRVM</t>
+          <t>&lt; B-</t>
         </is>
       </c>
       <c r="B99" s="13" t="inlineStr"/>
@@ -4979,31 +5411,23 @@
     <row r="100">
       <c r="A100" s="12" t="inlineStr">
         <is>
-          <t>Titre bancaire non noté</t>
+          <t>Non noté</t>
         </is>
       </c>
       <c r="B100" s="13" t="inlineStr"/>
     </row>
-    <row r="101">
-      <c r="A101" s="14" t="inlineStr">
-        <is>
-          <t>Action de l indice BRVM 10</t>
-        </is>
-      </c>
-      <c r="B101" s="13" t="inlineStr"/>
-    </row>
     <row r="102">
-      <c r="A102" s="12" t="inlineStr">
-        <is>
-          <t>Action d un indice principal reconnu</t>
-        </is>
-      </c>
-      <c r="B102" s="13" t="inlineStr"/>
+      <c r="A102" s="10" t="inlineStr">
+        <is>
+          <t>Type_emetteur (CRM financée)</t>
+        </is>
+      </c>
+      <c r="B102" s="11" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="14" t="inlineStr">
         <is>
-          <t>Autre action cotée à la BRVM ou sur une bourse reconnue</t>
+          <t>emprunteur souverain</t>
         </is>
       </c>
       <c r="B103" s="13" t="inlineStr"/>
@@ -5011,47 +5435,47 @@
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
         <is>
-          <t>Obligation convertible en action</t>
+          <t>autre émetteur</t>
         </is>
       </c>
       <c r="B104" s="13" t="inlineStr"/>
     </row>
-    <row r="105">
-      <c r="A105" s="14" t="inlineStr">
-        <is>
-          <t>OPCVM / FI</t>
-        </is>
-      </c>
-      <c r="B105" s="13" t="inlineStr"/>
-    </row>
     <row r="106">
-      <c r="A106" s="12" t="inlineStr">
-        <is>
-          <t>Panier d actifs</t>
-        </is>
-      </c>
-      <c r="B106" s="13" t="inlineStr"/>
+      <c r="A106" s="10" t="inlineStr">
+        <is>
+          <t>Maturite (CRM financée)</t>
+        </is>
+      </c>
+      <c r="B106" s="11" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="14" t="inlineStr">
         <is>
-          <t>Autre sûreté non éligible</t>
+          <t>&lt;=1 an</t>
         </is>
       </c>
       <c r="B107" s="13" t="inlineStr"/>
     </row>
+    <row r="108">
+      <c r="A108" s="12" t="inlineStr">
+        <is>
+          <t>1-3 ans</t>
+        </is>
+      </c>
+      <c r="B108" s="13" t="inlineStr"/>
+    </row>
     <row r="109">
-      <c r="A109" s="10" t="inlineStr">
-        <is>
-          <t>Cas_particulier_souverain (cascade : catégorie = Souverains)</t>
-        </is>
-      </c>
-      <c r="B109" s="11" t="inlineStr"/>
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t>3-5 ans</t>
+        </is>
+      </c>
+      <c r="B109" s="13" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="12" t="inlineStr">
         <is>
-          <t>Expositions sur États de l’UEMOA et démembrements libellées et financées en FCFA</t>
+          <t>5-10 ans</t>
         </is>
       </c>
       <c r="B110" s="13" t="inlineStr"/>
@@ -5059,31 +5483,23 @@
     <row r="111">
       <c r="A111" s="14" t="inlineStr">
         <is>
-          <t>Expositions sur BCEAO libellées et financées en FCFA</t>
+          <t>&gt;10 ans</t>
         </is>
       </c>
       <c r="B111" s="13" t="inlineStr"/>
     </row>
-    <row r="112">
-      <c r="A112" s="12" t="inlineStr">
-        <is>
-          <t>UEMOA</t>
-        </is>
-      </c>
-      <c r="B112" s="13" t="inlineStr"/>
-    </row>
     <row r="113">
-      <c r="A113" s="14" t="inlineStr">
-        <is>
-          <t>CEDEAO</t>
-        </is>
-      </c>
-      <c r="B113" s="13" t="inlineStr"/>
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>Type_Collatéral (CRM financée)</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="12" t="inlineStr">
         <is>
-          <t>UA</t>
+          <t>Liquidités dans la même devise</t>
         </is>
       </c>
       <c r="B114" s="13" t="inlineStr"/>
@@ -5091,7 +5507,7 @@
     <row r="115">
       <c r="A115" s="14" t="inlineStr">
         <is>
-          <t>UE</t>
+          <t>Liquidités dans une devise différente</t>
         </is>
       </c>
       <c r="B115" s="13" t="inlineStr"/>
@@ -5099,7 +5515,7 @@
     <row r="116">
       <c r="A116" s="12" t="inlineStr">
         <is>
-          <t>ONU</t>
+          <t>Or</t>
         </is>
       </c>
       <c r="B116" s="13" t="inlineStr"/>
@@ -5107,7 +5523,7 @@
     <row r="117">
       <c r="A117" s="14" t="inlineStr">
         <is>
-          <t>BRI</t>
+          <t>Titre de dette souverain</t>
         </is>
       </c>
       <c r="B117" s="13" t="inlineStr"/>
@@ -5115,7 +5531,7 @@
     <row r="118">
       <c r="A118" s="12" t="inlineStr">
         <is>
-          <t>FMI</t>
+          <t>Titre non noté émis par un État de l UMOA</t>
         </is>
       </c>
       <c r="B118" s="13" t="inlineStr"/>
@@ -5123,7 +5539,7 @@
     <row r="119">
       <c r="A119" s="14" t="inlineStr">
         <is>
-          <t>BCE</t>
+          <t>Titre de dette émis par un autre émetteur</t>
         </is>
       </c>
       <c r="B119" s="13" t="inlineStr"/>
@@ -5131,7 +5547,7 @@
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t>FGD-UMOA</t>
+          <t>Titre garanti par un agent agréé par la BRVM</t>
         </is>
       </c>
       <c r="B120" s="13" t="inlineStr"/>
@@ -5139,23 +5555,31 @@
     <row r="121">
       <c r="A121" s="14" t="inlineStr">
         <is>
-          <t>Aucun de ces cas</t>
+          <t>Titre bancaire non noté</t>
         </is>
       </c>
       <c r="B121" s="13" t="inlineStr"/>
     </row>
+    <row r="122">
+      <c r="A122" s="12" t="inlineStr">
+        <is>
+          <t>Action de l indice BRVM 10</t>
+        </is>
+      </c>
+      <c r="B122" s="13" t="inlineStr"/>
+    </row>
     <row r="123">
-      <c r="A123" s="10" t="inlineStr">
-        <is>
-          <t>Souverain_note_OCE (cascade : catégorie = Souverains)</t>
-        </is>
-      </c>
-      <c r="B123" s="11" t="inlineStr"/>
+      <c r="A123" s="14" t="inlineStr">
+        <is>
+          <t>Action d un indice principal reconnu</t>
+        </is>
+      </c>
+      <c r="B123" s="13" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Autre action cotée à la BRVM ou sur une bourse reconnue</t>
         </is>
       </c>
       <c r="B124" s="13" t="inlineStr"/>
@@ -5163,7 +5587,7 @@
     <row r="125">
       <c r="A125" s="14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Obligation convertible en action</t>
         </is>
       </c>
       <c r="B125" s="13" t="inlineStr"/>
@@ -5171,7 +5595,7 @@
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>OPCVM / FI</t>
         </is>
       </c>
       <c r="B126" s="13" t="inlineStr"/>
@@ -5179,7 +5603,7 @@
     <row r="127">
       <c r="A127" s="14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Panier d actifs</t>
         </is>
       </c>
       <c r="B127" s="13" t="inlineStr"/>
@@ -5187,91 +5611,87 @@
     <row r="128">
       <c r="A128" s="12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>Autre sûreté non éligible</t>
         </is>
       </c>
       <c r="B128" s="13" t="inlineStr"/>
     </row>
-    <row r="129">
-      <c r="A129" s="14" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B129" s="13" t="inlineStr"/>
-    </row>
     <row r="130">
-      <c r="A130" s="12" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B130" s="13" t="inlineStr"/>
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>Cas_particulier_souverain</t>
+        </is>
+      </c>
+      <c r="B130" s="11" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="14" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>Expositions sur États de l’UEMOA et démembrements libellées et financées en FCFA</t>
         </is>
       </c>
       <c r="B131" s="13" t="inlineStr"/>
     </row>
+    <row r="132">
+      <c r="A132" s="12" t="inlineStr">
+        <is>
+          <t>Expositions sur BCEAO libellées et financées en FCFA</t>
+        </is>
+      </c>
+      <c r="B132" s="13" t="inlineStr"/>
+    </row>
     <row r="133">
-      <c r="A133" s="10" t="inlineStr">
-        <is>
-          <t>Cas_institution_bancaire (cascade : catégorie = Institutions financières)</t>
-        </is>
-      </c>
-      <c r="B133" s="11" t="inlineStr"/>
+      <c r="A133" s="14" t="inlineStr">
+        <is>
+          <t>UEMOA</t>
+        </is>
+      </c>
+      <c r="B133" s="13" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
         <is>
-          <t>equivalent_umoa_rules</t>
-        </is>
-      </c>
-      <c r="B134" s="13" t="inlineStr">
-        <is>
-          <t>Banque hors UMOA soumise à des règles équivalentes à celles de l'UMOA</t>
-        </is>
-      </c>
+          <t>CEDEAO</t>
+        </is>
+      </c>
+      <c r="B134" s="13" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="14" t="inlineStr">
         <is>
-          <t>weak_prudential_case</t>
-        </is>
-      </c>
-      <c r="B135" s="13" t="inlineStr">
-        <is>
-          <t>Banque en difficulté prudentielle</t>
-        </is>
-      </c>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="B135" s="13" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
         <is>
-          <t>eligible_categories_case</t>
-        </is>
-      </c>
-      <c r="B136" s="13" t="inlineStr">
-        <is>
-          <t>Institution faisant partie des catégories éligibles (voir notation)</t>
-        </is>
-      </c>
+          <t>UE</t>
+        </is>
+      </c>
+      <c r="B136" s="13" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="14" t="inlineStr">
+        <is>
+          <t>ONU</t>
+        </is>
+      </c>
+      <c r="B137" s="13" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" s="10" t="inlineStr">
-        <is>
-          <t>Type_autre_actif (cascade : catégorie = Autres actifs)</t>
-        </is>
-      </c>
-      <c r="B138" s="11" t="inlineStr"/>
+      <c r="A138" s="12" t="inlineStr">
+        <is>
+          <t>BRI</t>
+        </is>
+      </c>
+      <c r="B138" s="13" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="14" t="inlineStr">
         <is>
-          <t>Encaisse</t>
+          <t>FMI</t>
         </is>
       </c>
       <c r="B139" s="13" t="inlineStr"/>
@@ -5279,7 +5699,7 @@
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t>Valeurs assimilées à l’encaisse, y compris l’or</t>
+          <t>BCE</t>
         </is>
       </c>
       <c r="B140" s="13" t="inlineStr"/>
@@ -5287,7 +5707,7 @@
     <row r="141">
       <c r="A141" s="14" t="inlineStr">
         <is>
-          <t>Valeurs à l’encaissement avec crédit immédiat</t>
+          <t>FGD-UMOA</t>
         </is>
       </c>
       <c r="B141" s="13" t="inlineStr"/>
@@ -5295,31 +5715,23 @@
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t>Participations non significatives non déduites des fonds propres</t>
+          <t>Aucun de ces cas</t>
         </is>
       </c>
       <c r="B142" s="13" t="inlineStr"/>
     </row>
-    <row r="143">
-      <c r="A143" s="14" t="inlineStr">
-        <is>
-          <t>Immobilisations corporelles</t>
-        </is>
-      </c>
-      <c r="B143" s="13" t="inlineStr"/>
-    </row>
     <row r="144">
-      <c r="A144" s="12" t="inlineStr">
-        <is>
-          <t>Immobilisations hors exploitation</t>
-        </is>
-      </c>
-      <c r="B144" s="13" t="inlineStr"/>
+      <c r="A144" s="10" t="inlineStr">
+        <is>
+          <t>Souverain_note_OCE</t>
+        </is>
+      </c>
+      <c r="B144" s="11" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="14" t="inlineStr">
         <is>
-          <t>Immobilisations incorporelles</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B145" s="13" t="inlineStr"/>
@@ -5327,7 +5739,7 @@
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
-          <t>Autres actifs divers</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B146" s="13" t="inlineStr"/>
@@ -5335,7 +5747,7 @@
     <row r="147">
       <c r="A147" s="14" t="inlineStr">
         <is>
-          <t>Engagements en actions non déduits</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B147" s="13" t="inlineStr"/>
@@ -5343,7 +5755,7 @@
     <row r="148">
       <c r="A148" s="12" t="inlineStr">
         <is>
-          <t>Expositions sur entreprises financières non soumises à une réglementation équivalente UMOA</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B148" s="13" t="inlineStr"/>
@@ -5351,7 +5763,7 @@
     <row r="149">
       <c r="A149" s="14" t="inlineStr">
         <is>
-          <t>Autres éléments d’actifs non définis</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B149" s="13" t="inlineStr"/>
@@ -5359,7 +5771,7 @@
     <row r="150">
       <c r="A150" s="12" t="inlineStr">
         <is>
-          <t>Participations significatives et impôts différés actifs non déduits</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B150" s="13" t="inlineStr"/>
@@ -5367,116 +5779,432 @@
     <row r="151">
       <c r="A151" s="14" t="inlineStr">
         <is>
-          <t>Expositions sur établissements non conformes aux ratios de solvabilité</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B151" s="13" t="inlineStr"/>
     </row>
-    <row r="153">
-      <c r="A153" s="10" t="inlineStr">
-        <is>
-          <t>Ponderation_initiale_avant_defaut (cascade : catégorie = Créances en souffrance)</t>
-        </is>
-      </c>
-      <c r="B153" s="11" t="inlineStr"/>
+    <row r="152">
+      <c r="A152" s="12" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B152" s="13" t="inlineStr"/>
     </row>
     <row r="154">
-      <c r="A154" s="12" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="B154" s="13" t="inlineStr"/>
+      <c r="A154" s="10" t="inlineStr">
+        <is>
+          <t>Cas_organisme_public</t>
+        </is>
+      </c>
+      <c r="B154" s="11" t="inlineStr"/>
     </row>
     <row r="155">
-      <c r="A155" s="14" t="n">
-        <v>0.35</v>
+      <c r="A155" s="14" t="inlineStr">
+        <is>
+          <t>Organisme public standard (selon notation)</t>
+        </is>
       </c>
       <c r="B155" s="13" t="inlineStr"/>
     </row>
     <row r="156">
-      <c r="A156" s="12" t="n">
-        <v>0.5</v>
+      <c r="A156" s="12" t="inlineStr">
+        <is>
+          <t>Organisme public UEMOA libellé en FCFA (préférentiel 20%)</t>
+        </is>
       </c>
       <c r="B156" s="13" t="inlineStr"/>
     </row>
     <row r="157">
-      <c r="A157" s="14" t="n">
-        <v>0.75</v>
+      <c r="A157" s="14" t="inlineStr">
+        <is>
+          <t>Activité commerciale / non publique (traité comme entreprise)</t>
+        </is>
       </c>
       <c r="B157" s="13" t="inlineStr"/>
     </row>
-    <row r="158">
-      <c r="A158" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="B158" s="13" t="inlineStr"/>
-    </row>
     <row r="159">
-      <c r="A159" s="14" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="B159" s="13" t="inlineStr"/>
+      <c r="A159" s="10" t="inlineStr">
+        <is>
+          <t>Cas_particulier_bmd</t>
+        </is>
+      </c>
+      <c r="B159" s="11" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160" s="12" t="n">
-        <v>2.5</v>
+      <c r="A160" s="12" t="inlineStr">
+        <is>
+          <t>BMD standard (selon notation)</t>
+        </is>
       </c>
       <c r="B160" s="13" t="inlineStr"/>
     </row>
+    <row r="161">
+      <c r="A161" s="14" t="inlineStr">
+        <is>
+          <t>BMD haute qualité / soutien fort (pondération 0%)</t>
+        </is>
+      </c>
+      <c r="B161" s="13" t="inlineStr"/>
+    </row>
     <row r="162">
-      <c r="A162" s="10" t="inlineStr">
-        <is>
-          <t>Devise / Devise_Collatéral</t>
-        </is>
-      </c>
-      <c r="B162" s="11" t="inlineStr"/>
+      <c r="A162" s="12" t="inlineStr">
+        <is>
+          <t>BMD institution listée BCEAO en FCFA (BIRD, BAD, BOAD... 0%)</t>
+        </is>
+      </c>
+      <c r="B162" s="13" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="14" t="inlineStr">
         <is>
-          <t>XOF</t>
+          <t>BMD UEMOA en FCFA conforme aux critères (20%)</t>
         </is>
       </c>
       <c r="B163" s="13" t="inlineStr"/>
     </row>
-    <row r="164">
-      <c r="A164" s="12" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="B164" s="13" t="inlineStr"/>
-    </row>
     <row r="165">
-      <c r="A165" s="14" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="B165" s="13" t="inlineStr"/>
+      <c r="A165" s="10" t="inlineStr">
+        <is>
+          <t>Cas_institution_bancaire</t>
+        </is>
+      </c>
+      <c r="B165" s="11" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="12" t="inlineStr">
+        <is>
+          <t>equivalent_umoa_rules</t>
+        </is>
+      </c>
+      <c r="B166" s="13" t="inlineStr">
+        <is>
+          <t>Banque hors UMOA soumise à des règles équivalentes à celles de l'UMOA</t>
+        </is>
+      </c>
     </row>
     <row r="167">
-      <c r="A167" s="10" t="inlineStr">
-        <is>
-          <t>Champs Oui/Non (tous les Souverain_*, BMD_*, Organisme_public_*, Clientele_detail_*, Immobilier_*, Defaut_*, Entreprise_*, Obligation_convertible_indice_principal) — la plupart sont en cascade selon Catégorie d'exposition, voir l'onglet Instructions</t>
-        </is>
-      </c>
-      <c r="B167" s="11" t="inlineStr"/>
+      <c r="A167" s="14" t="inlineStr">
+        <is>
+          <t>weak_prudential_case</t>
+        </is>
+      </c>
+      <c r="B167" s="13" t="inlineStr">
+        <is>
+          <t>Banque en difficulté prudentielle</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="12" t="inlineStr">
         <is>
+          <t>eligible_categories_case</t>
+        </is>
+      </c>
+      <c r="B168" s="13" t="inlineStr">
+        <is>
+          <t>Institution faisant partie des catégories éligibles (voir notation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="10" t="inlineStr">
+        <is>
+          <t>Type_autre_actif</t>
+        </is>
+      </c>
+      <c r="B170" s="11" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="14" t="inlineStr">
+        <is>
+          <t>Encaisse</t>
+        </is>
+      </c>
+      <c r="B171" s="13" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="12" t="inlineStr">
+        <is>
+          <t>Valeurs assimilées à l’encaisse, y compris l’or</t>
+        </is>
+      </c>
+      <c r="B172" s="13" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="14" t="inlineStr">
+        <is>
+          <t>Valeurs à l’encaissement avec crédit immédiat</t>
+        </is>
+      </c>
+      <c r="B173" s="13" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="12" t="inlineStr">
+        <is>
+          <t>Participations non significatives non déduites des fonds propres</t>
+        </is>
+      </c>
+      <c r="B174" s="13" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="14" t="inlineStr">
+        <is>
+          <t>Immobilisations corporelles</t>
+        </is>
+      </c>
+      <c r="B175" s="13" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="12" t="inlineStr">
+        <is>
+          <t>Immobilisations hors exploitation</t>
+        </is>
+      </c>
+      <c r="B176" s="13" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="14" t="inlineStr">
+        <is>
+          <t>Immobilisations incorporelles</t>
+        </is>
+      </c>
+      <c r="B177" s="13" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="12" t="inlineStr">
+        <is>
+          <t>Autres actifs divers</t>
+        </is>
+      </c>
+      <c r="B178" s="13" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="14" t="inlineStr">
+        <is>
+          <t>Engagements en actions non déduits</t>
+        </is>
+      </c>
+      <c r="B179" s="13" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="12" t="inlineStr">
+        <is>
+          <t>Expositions sur entreprises financières non soumises à une réglementation équivalente UMOA</t>
+        </is>
+      </c>
+      <c r="B180" s="13" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="14" t="inlineStr">
+        <is>
+          <t>Autres éléments d’actifs non définis</t>
+        </is>
+      </c>
+      <c r="B181" s="13" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="12" t="inlineStr">
+        <is>
+          <t>Participations significatives et impôts différés actifs non déduits</t>
+        </is>
+      </c>
+      <c r="B182" s="13" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="14" t="inlineStr">
+        <is>
+          <t>Expositions sur établissements non conformes aux ratios de solvabilité</t>
+        </is>
+      </c>
+      <c r="B183" s="13" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="10" t="inlineStr">
+        <is>
+          <t>Cas_creance_souffrance</t>
+        </is>
+      </c>
+      <c r="B185" s="11" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="12" t="inlineStr">
+        <is>
+          <t>Prêt immobilier résidentiel en défaut (Provisions &gt;= 20%) — 50%</t>
+        </is>
+      </c>
+      <c r="B186" s="13" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="14" t="inlineStr">
+        <is>
+          <t>Prêt immobilier résidentiel en défaut (Provisions &lt; 20%) — 100%</t>
+        </is>
+      </c>
+      <c r="B187" s="13" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="12" t="inlineStr">
+        <is>
+          <t>Autre créance en défaut (Provisions &gt;= 20%) — 100%</t>
+        </is>
+      </c>
+      <c r="B188" s="13" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="14" t="inlineStr">
+        <is>
+          <t>Autre créance en défaut (Provisions &lt; 20%) — 150%</t>
+        </is>
+      </c>
+      <c r="B189" s="13" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="10" t="inlineStr">
+        <is>
+          <t>Cas_particulier_entreprise</t>
+        </is>
+      </c>
+      <c r="B191" s="11" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="12" t="inlineStr">
+        <is>
+          <t>Entreprise standard (selon notation ou 100%)</t>
+        </is>
+      </c>
+      <c r="B192" s="13" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="14" t="inlineStr">
+        <is>
+          <t>Portefeuille dégradé (seuil BCEAO dépassé -&gt; 150%)</t>
+        </is>
+      </c>
+      <c r="B193" s="13" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="12" t="inlineStr">
+        <is>
+          <t>Entreprise faisant l'objet d'une procédure prudentielle</t>
+        </is>
+      </c>
+      <c r="B194" s="13" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="14" t="inlineStr">
+        <is>
+          <t>Entreprise d'investissement non soumise à la loi bancaire (100%)</t>
+        </is>
+      </c>
+      <c r="B195" s="13" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="10" t="inlineStr">
+        <is>
+          <t>Ponderation_initiale_avant_defaut</t>
+        </is>
+      </c>
+      <c r="B197" s="11" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B198" s="13" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="14" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B199" s="13" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B200" s="13" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="14" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="B201" s="13" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B202" s="13" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="14" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B203" s="13" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B204" s="13" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="10" t="inlineStr">
+        <is>
+          <t>Devise / Devise_Collatéral</t>
+        </is>
+      </c>
+      <c r="B206" s="11" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="14" t="inlineStr">
+        <is>
+          <t>XOF</t>
+        </is>
+      </c>
+      <c r="B207" s="13" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="12" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="B208" s="13" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="14" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B209" s="13" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="10" t="inlineStr">
+        <is>
+          <t>Champs Oui/Non (Souverain_*, Clientele_detail_*, Immobilier_*, Obligation_convertible_indice_principal)</t>
+        </is>
+      </c>
+      <c r="B211" s="11" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="12" t="inlineStr">
+        <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="B168" s="13" t="inlineStr"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="14" t="inlineStr">
+      <c r="B212" s="13" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="14" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="B169" s="13" t="inlineStr"/>
+      <c r="B213" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>